<commit_message>
RC-is-good but BOL needs excel template
</commit_message>
<xml_diff>
--- a/RC-template.xlsx
+++ b/RC-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ew-josh/Downloads/EW-Design/EW-WebView/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84929075-A8EB-9E4F-803C-92959494607E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{053AF822-1E99-AF47-BDFA-C65D1D37C776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38400" yWindow="12680" windowWidth="28800" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t xml:space="preserve">Carrier Rate Confirmation        </t>
   </si>
@@ -185,12 +185,6 @@
   </si>
   <si>
     <t xml:space="preserve">Load Information: </t>
-  </si>
-  <si>
-    <t>drop off ：</t>
-  </si>
-  <si>
-    <t>Pick up：</t>
   </si>
 </sst>
 </file>
@@ -544,6 +538,30 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -588,30 +606,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1023,13 +1017,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" s="1" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
       <c r="F1" s="9" t="s">
         <v>2</v>
       </c>
@@ -1043,94 +1037,90 @@
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
-      <c r="F2" s="29" t="s">
+      <c r="F2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
     </row>
     <row r="3" spans="1:9" ht="94.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="30" t="s">
+      <c r="A3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31" t="s">
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="G3" s="32"/>
-      <c r="H3" s="32"/>
-      <c r="I3" s="32"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+      <c r="I3" s="17"/>
     </row>
     <row r="4" spans="1:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="34"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="34"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="35"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="20"/>
     </row>
     <row r="5" spans="1:9" s="1" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="18"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="26"/>
     </row>
     <row r="6" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="21"/>
+      <c r="A6" s="27"/>
+      <c r="B6" s="28"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="29"/>
     </row>
     <row r="7" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="26"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="27"/>
+      <c r="A7" s="33"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="34"/>
+      <c r="E7" s="34"/>
+      <c r="F7" s="34"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="35"/>
     </row>
     <row r="8" spans="1:9" ht="14" x14ac:dyDescent="0.2">
       <c r="A8" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="C8" s="22"/>
-      <c r="D8" s="22"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="23" t="s">
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="G8" s="24"/>
+      <c r="G8" s="32"/>
       <c r="H8" s="12" t="s">
         <v>5</v>
       </c>
@@ -1140,12 +1130,12 @@
     </row>
     <row r="9" spans="1:9" s="1" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
       <c r="H9" s="6"/>
       <c r="I9" s="7"/>
     </row>
@@ -1163,17 +1153,17 @@
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:9" s="2" customFormat="1" ht="26.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
-      <c r="H11" s="15"/>
-      <c r="I11" s="15"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
     </row>
     <row r="12" spans="1:9" s="2" customFormat="1" ht="96" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="3"/>
@@ -1188,11 +1178,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="A4:I4"/>
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="A11:I11"/>
@@ -1201,6 +1186,11 @@
     <mergeCell ref="B8:E8"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="A7:I7"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="A4:I4"/>
   </mergeCells>
   <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>

</xml_diff>